<commit_message>
MainPLC: CAN gateway, Modbus RTU doors poll, web page; display doors block; firmware update concept; docs and web configurator
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Docs/Project_Costs.xlsx
+++ b/Docs/Project_Costs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\morfe\STM32CubeIDE\workspace_1.17.0\HVAC_CleanRoom_Project\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AB3A0CC-7657-4D87-9FA6-A297188B5A43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1709863-7257-4908-813E-EAFA5EFF8D15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -84,7 +84,88 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="89">
+  <si>
+    <t>№</t>
+  </si>
+  <si>
+    <t>Артикул</t>
+  </si>
+  <si>
+    <t>Наименование</t>
+  </si>
+  <si>
+    <t>Цена партии</t>
+  </si>
+  <si>
+    <t>Кол-во в партии</t>
+  </si>
+  <si>
+    <t>Цена за ед.</t>
+  </si>
+  <si>
+    <t>Доставка</t>
+  </si>
+  <si>
+    <t>Кол-во на модуль</t>
+  </si>
+  <si>
+    <t>Сумма</t>
+  </si>
+  <si>
+    <t>Корпус</t>
+  </si>
+  <si>
+    <t>2896241</t>
+  </si>
+  <si>
+    <t>Нижняя часть корпуса (BC 17,8 UT HBUS BK)</t>
+  </si>
+  <si>
+    <t>2279732</t>
+  </si>
+  <si>
+    <t>Верхняя часть корпуса (BC 17,8 OTU MKDSO KMGY)</t>
+  </si>
+  <si>
+    <t>Клеммный блок на плату (MKDSO 1,5/ 4-L-3,5 KMGY)</t>
+  </si>
+  <si>
+    <t>Заглушка (ME B-17,5 MKDSO KMGY)</t>
+  </si>
+  <si>
+    <t>2896102</t>
+  </si>
+  <si>
+    <t>Прозрачная крышка корпуса (BC 17,8 DKL S TRANS)</t>
+  </si>
+  <si>
+    <t>2896322</t>
+  </si>
+  <si>
+    <t>Шинный соединитель на DIN-рейку (HBUS 53,6-16P-3S BK)</t>
+  </si>
+  <si>
+    <t>Идет один на ри модуля</t>
+  </si>
+  <si>
+    <t>Итого корпус</t>
+  </si>
+  <si>
+    <t>Плата</t>
+  </si>
+  <si>
+    <t>SMT026082260698-Y214</t>
+  </si>
+  <si>
+    <t>Печатная плата в сборе Modul_AI</t>
+  </si>
+  <si>
+    <t>Итого плата</t>
+  </si>
+  <si>
+    <t>Всего модуль</t>
+  </si>
   <si>
     <t>Номер заказа</t>
   </si>
@@ -137,7 +218,10 @@
     <t>JLCPCB</t>
   </si>
   <si>
-    <t>Артикул</t>
+    <t>440482</t>
+  </si>
+  <si>
+    <t>08/09/2026</t>
   </si>
   <si>
     <t>Описание</t>
@@ -149,12 +233,12 @@
     <t>Количество</t>
   </si>
   <si>
+    <t>Цена за шт (EUR/DOL)</t>
+  </si>
+  <si>
     <t>Итого (ILS)</t>
   </si>
   <si>
-    <t>2896241</t>
-  </si>
-  <si>
     <t>BC 17,8 UT HBUS BK</t>
   </si>
   <si>
@@ -170,9 +254,6 @@
     <t>Крышка корпуса</t>
   </si>
   <si>
-    <t>2896322</t>
-  </si>
-  <si>
     <t>HBUS 53,6-16P-3S BK</t>
   </si>
   <si>
@@ -206,9 +287,6 @@
     <t>Штыревой разъем (гребенка)</t>
   </si>
   <si>
-    <t>2279732</t>
-  </si>
-  <si>
     <t>BC 17,8 OTU MKDSO KMGY</t>
   </si>
   <si>
@@ -221,7 +299,7 @@
     <t>HBUS 35,6-16P-1S BK</t>
   </si>
   <si>
-    <t>2896102</t>
+    <t>183969, 440482</t>
   </si>
   <si>
     <t>BC 17,8 DKL S TRANS</t>
@@ -269,79 +347,10 @@
     <t>BC 35,6 DKL S TRANS</t>
   </si>
   <si>
-    <t>SMT026082260698-Y214</t>
-  </si>
-  <si>
     <t>Rigid Populated printed circuit board (Modul_AI)</t>
   </si>
   <si>
     <t>Печатная плата в сборе</t>
-  </si>
-  <si>
-    <t>№</t>
-  </si>
-  <si>
-    <t>Наименование</t>
-  </si>
-  <si>
-    <t>Цена партии</t>
-  </si>
-  <si>
-    <t>Кол-во в партии</t>
-  </si>
-  <si>
-    <t>Цена за ед.</t>
-  </si>
-  <si>
-    <t>Доставка</t>
-  </si>
-  <si>
-    <t>Кол-во на модуль</t>
-  </si>
-  <si>
-    <t>Сумма</t>
-  </si>
-  <si>
-    <t>Корпус</t>
-  </si>
-  <si>
-    <t>Нижняя часть корпуса (BC 17,8 UT HBUS BK)</t>
-  </si>
-  <si>
-    <t>Верхняя часть корпуса (BC 17,8 OTU MKDSO KMGY)</t>
-  </si>
-  <si>
-    <t>Клеммный блок на плату (MKDSO 1,5/ 4-L-3,5 KMGY)</t>
-  </si>
-  <si>
-    <t>Заглушка (ME B-17,5 MKDSO KMGY)</t>
-  </si>
-  <si>
-    <t>Прозрачная крышка корпуса (BC 17,8 DKL S TRANS)</t>
-  </si>
-  <si>
-    <t>Шинный соединитель на DIN-рейку (HBUS 53,6-16P-3S BK)</t>
-  </si>
-  <si>
-    <t>Итого корпус</t>
-  </si>
-  <si>
-    <t>Плата</t>
-  </si>
-  <si>
-    <t>Печатная плата в сборе Modul_AI</t>
-  </si>
-  <si>
-    <t>Итого плата</t>
-  </si>
-  <si>
-    <t>Всего модуль</t>
-  </si>
-  <si>
-    <t>Цена за шт (EUR/DOL)</t>
-  </si>
-  <si>
-    <t>Идет один на ри модуля</t>
   </si>
 </sst>
 </file>
@@ -465,7 +474,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -542,11 +551,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -584,12 +606,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -608,6 +624,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -618,13 +637,25 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -761,20 +792,17 @@
     <v>3</v>
     <v>Finance</v>
     <v>4</v>
-    <v>3.4211999999999998</v>
+    <v>3.3700999999999999</v>
     <v>2.7978000000000001</v>
-    <v>1.35E-2</v>
-    <v>4.5199999999999997E-3</v>
+    <v>-1.72E-2</v>
+    <v>-5.6439999999999997E-3</v>
     <v>ILS</v>
     <v>USD</v>
-    <v>3.0024000000000002</v>
     <v>Currency Pair</v>
-    <v>46258.690057870372</v>
-    <v>2.9832000000000001</v>
+    <v>46276.873796296299</v>
     <v>US Dollar/Israeli Shekel FX Spot Rate</v>
-    <v>2.9866999999999999</v>
-    <v>2.9864999999999999</v>
-    <v>3</v>
+    <v>3.0476000000000001</v>
+    <v>3.0304000000000002</v>
     <v>USDILS</v>
     <v>USD/ILS</v>
   </rv>
@@ -793,20 +821,17 @@
     <v>3</v>
     <v>Finance</v>
     <v>4</v>
-    <v>3.9851999999999999</v>
+    <v>3.9706999999999999</v>
     <v>3.2562000000000002</v>
-    <v>1.1599999999999999E-2</v>
-    <v>3.3250000000000003E-3</v>
+    <v>-2.3599999999999999E-2</v>
+    <v>-6.6700000000000006E-3</v>
     <v>ILS</v>
     <v>EUR</v>
-    <v>3.5028999999999999</v>
     <v>Currency Pair</v>
-    <v>46258.690069444441</v>
-    <v>3.4857999999999998</v>
+    <v>46276.874652777777</v>
     <v>Euro/Israeli Shekel FX Cross Rate</v>
-    <v>3.4855</v>
-    <v>3.4882</v>
-    <v>3.4998</v>
+    <v>3.5383</v>
+    <v>3.5146999999999999</v>
     <v>EURILS</v>
     <v>EUR/ILS</v>
   </rv>
@@ -836,12 +861,9 @@
     <k n="Change (%)"/>
     <k n="Currency" t="s"/>
     <k n="From currency" t="s"/>
-    <k n="High"/>
     <k n="Instrument type" t="s"/>
     <k n="Last trade time"/>
-    <k n="Low"/>
     <k n="Name" t="s"/>
-    <k n="Open"/>
     <k n="Previous close"/>
     <k n="Price"/>
     <k n="Ticker symbol" t="s"/>
@@ -856,7 +878,7 @@
 <file path=xl/richData/rdsupportingpropertybag.xml><?xml version="1.0" encoding="utf-8"?>
 <supportingPropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2">
   <spbArrays count="1">
-    <a count="27">
+    <a count="24">
       <v t="s">%EntityServiceId</v>
       <v t="s">_Format</v>
       <v t="s">%IsRefreshable</v>
@@ -874,9 +896,6 @@
       <v t="s">Currency</v>
       <v t="s">From currency</v>
       <v t="s">Previous close</v>
-      <v t="s">Open</v>
-      <v t="s">High</v>
-      <v t="s">Low</v>
       <v t="s">52 week high</v>
       <v t="s">52 week low</v>
       <v t="s">Instrument type</v>
@@ -902,15 +921,12 @@
     </spb>
     <spb s="3">
       <v>1</v>
-      <v>1</v>
       <v>2</v>
-      <v>1</v>
-      <v>1</v>
-      <v>1</v>
+      <v>2</v>
       <v>3</v>
-      <v>1</v>
-      <v>1</v>
-      <v>1</v>
+      <v>2</v>
+      <v>2</v>
+      <v>2</v>
       <v>4</v>
       <v>5</v>
     </spb>
@@ -937,10 +953,7 @@
     <k n="`%ProviderInfo" t="spb"/>
   </s>
   <s>
-    <k n="Low" t="i"/>
-    <k n="High" t="i"/>
     <k n="Name" t="i"/>
-    <k n="Open" t="i"/>
     <k n="Price" t="i"/>
     <k n="Change" t="i"/>
     <k n="Change (%)" t="i"/>
@@ -973,20 +986,20 @@
     </x:dxf>
   </dxfs>
   <richProperties>
+    <rPr n="IsTitleField" t="b"/>
     <rPr n="NumberFormat" t="s"/>
-    <rPr n="IsTitleField" t="b"/>
   </richProperties>
   <richStyles>
+    <rSty>
+      <rpv i="0">1</rpv>
+    </rSty>
     <rSty dxfid="0">
-      <rpv i="0" xml:space="preserve">_ [$₪-he-IL] * #,##0.00_ ;_ [$₪-he-IL] * -#,##0.00_ ;_ [$₪-he-IL] * "-"??_ ;_ @_ </rpv>
-    </rSty>
-    <rSty>
-      <rpv i="1">1</rpv>
+      <rpv i="1" xml:space="preserve">_ [$₪-he-IL] * #,##0.00_ ;_ [$₪-he-IL] * -#,##0.00_ ;_ [$₪-he-IL] * "-"??_ ;_ @_ </rpv>
     </rSty>
     <rSty dxfid="1"/>
     <rSty dxfid="2"/>
     <rSty dxfid="3">
-      <rpv i="0">0.00</rpv>
+      <rpv i="1">0.00</rpv>
     </rSty>
   </richStyles>
 </richStyleSheet>
@@ -1277,144 +1290,173 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" style="13" customWidth="1"/>
     <col min="2" max="2" width="13" style="13" customWidth="1"/>
-    <col min="3" max="3" width="18" style="16" customWidth="1"/>
-    <col min="4" max="4" width="22" style="13" customWidth="1"/>
-    <col min="5" max="5" width="12" style="13" customWidth="1"/>
-    <col min="6" max="6" width="20" style="13" customWidth="1"/>
-    <col min="7" max="7" width="17" style="13" customWidth="1"/>
-    <col min="8" max="8" width="19" style="13" customWidth="1"/>
+    <col min="3" max="3" width="18" style="33" customWidth="1"/>
+    <col min="4" max="4" width="22" style="33" customWidth="1"/>
+    <col min="5" max="5" width="12" style="33" customWidth="1"/>
+    <col min="6" max="6" width="20" style="33" customWidth="1"/>
+    <col min="7" max="7" width="17" style="33" customWidth="1"/>
+    <col min="8" max="8" width="19" style="33" customWidth="1"/>
     <col min="11" max="11" width="13.33203125" customWidth="1"/>
     <col min="12" max="12" width="14.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="14" t="s">
-        <v>2</v>
+        <v>28</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>29</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="K1" s="29" t="s">
-        <v>8</v>
-      </c>
-      <c r="L1" s="29"/>
-    </row>
-    <row r="2" spans="1:12" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+      <c r="L1" s="30"/>
+    </row>
+    <row r="2" spans="1:12" ht="21" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" s="12">
+        <v>37</v>
+      </c>
+      <c r="C2" s="32" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="34">
         <v>1815.8</v>
       </c>
-      <c r="E2" s="12">
+      <c r="E2" s="34">
         <v>326.83999999999997</v>
       </c>
-      <c r="F2" s="12">
+      <c r="F2" s="34">
         <v>2142.64</v>
       </c>
-      <c r="G2" s="12">
-        <v>0</v>
-      </c>
-      <c r="H2" s="12">
-        <v>0</v>
-      </c>
-      <c r="K2" s="17" t="e" vm="1">
+      <c r="G2" s="34">
+        <v>0</v>
+      </c>
+      <c r="H2" s="34">
+        <v>0</v>
+      </c>
+      <c r="K2" s="15" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="L2" s="18" cm="1">
+      <c r="L2" s="16" cm="1">
         <f t="array" aca="1" ref="L2" ca="1">_FV(K2,"Price")</f>
-        <v>3</v>
+        <v>3.0304000000000002</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="12" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="12">
+        <v>40</v>
+      </c>
+      <c r="C3" s="32" t="s">
+        <v>38</v>
+      </c>
+      <c r="D3" s="34">
         <v>825.96</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="34">
         <v>148.66999999999999</v>
       </c>
-      <c r="F3" s="12">
+      <c r="F3" s="34">
         <v>974.63</v>
       </c>
-      <c r="G3" s="12">
-        <v>0</v>
-      </c>
-      <c r="H3" s="12">
-        <v>0</v>
-      </c>
-      <c r="K3" s="17" t="e" vm="2">
+      <c r="G3" s="34">
+        <v>0</v>
+      </c>
+      <c r="H3" s="34">
+        <v>0</v>
+      </c>
+      <c r="K3" s="15" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="L3" s="19" cm="1">
+      <c r="L3" s="17" cm="1">
         <f t="array" aca="1" ref="L3" ca="1">_FV(K3,"Price")</f>
-        <v>3.4998</v>
+        <v>3.5146999999999999</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="20">
+        <v>42</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" s="18">
         <f ca="1">156.07*L2</f>
-        <v>468.21</v>
-      </c>
-      <c r="E4" s="10">
-        <v>0</v>
-      </c>
-      <c r="F4" s="20">
+        <v>472.95452800000004</v>
+      </c>
+      <c r="E4" s="18">
+        <v>0</v>
+      </c>
+      <c r="F4" s="18">
         <f ca="1">156.07*L2</f>
-        <v>468.21</v>
-      </c>
-      <c r="G4" s="20">
+        <v>472.95452800000004</v>
+      </c>
+      <c r="G4" s="18">
         <f ca="1">25.29*L2</f>
-        <v>75.87</v>
-      </c>
-      <c r="H4" s="10">
-        <v>0</v>
+        <v>76.638816000000006</v>
+      </c>
+      <c r="H4" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" s="31" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" s="18">
+        <v>488.98</v>
+      </c>
+      <c r="E5" s="18">
+        <v>88.02</v>
+      </c>
+      <c r="F5" s="18">
+        <v>577</v>
+      </c>
+      <c r="G5" s="18">
+        <v>0</v>
+      </c>
+      <c r="H5" s="18">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>3.5015000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -1422,6 +1464,7 @@
     <mergeCell ref="K1:L1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1430,7 +1473,7 @@
   <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.21875" style="22" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.21875" style="20" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="40.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="32.33203125" bestFit="1" customWidth="1"/>
@@ -1441,39 +1484,39 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="14" t="s">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>84</v>
+        <v>49</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="21" t="s">
-        <v>9</v>
+      <c r="A2" s="19" t="s">
+        <v>36</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="E2" s="12">
         <v>10</v>
@@ -1486,17 +1529,17 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="21" t="s">
-        <v>9</v>
+      <c r="A3" s="19" t="s">
+        <v>36</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>26</v>
+        <v>54</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="E3" s="12">
         <v>10</v>
@@ -1509,17 +1552,17 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="21" t="s">
-        <v>9</v>
+      <c r="A4" s="19" t="s">
+        <v>36</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>29</v>
+        <v>56</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>30</v>
+        <v>57</v>
       </c>
       <c r="E4" s="12">
         <v>10</v>
@@ -1532,17 +1575,17 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="21" t="s">
-        <v>9</v>
+      <c r="A5" s="19" t="s">
+        <v>36</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>31</v>
+        <v>58</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>32</v>
+        <v>59</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="E5" s="12">
         <v>50</v>
@@ -1555,17 +1598,17 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="21" t="s">
-        <v>9</v>
+      <c r="A6" s="19" t="s">
+        <v>36</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>34</v>
+        <v>61</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>35</v>
+        <v>62</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>36</v>
+        <v>63</v>
       </c>
       <c r="E6" s="12">
         <v>50</v>
@@ -1578,17 +1621,17 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="21" t="s">
-        <v>9</v>
+      <c r="A7" s="19" t="s">
+        <v>36</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>37</v>
+        <v>64</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>38</v>
+        <v>65</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>39</v>
+        <v>66</v>
       </c>
       <c r="E7" s="12">
         <v>50</v>
@@ -1601,17 +1644,17 @@
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="21" t="s">
-        <v>9</v>
+      <c r="A8" s="19" t="s">
+        <v>36</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>41</v>
+        <v>67</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>42</v>
+        <v>68</v>
       </c>
       <c r="E8" s="12">
         <v>10</v>
@@ -1624,17 +1667,17 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="21" t="s">
-        <v>9</v>
+      <c r="A9" s="19" t="s">
+        <v>36</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>43</v>
+        <v>69</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>44</v>
+        <v>70</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>30</v>
+        <v>57</v>
       </c>
       <c r="E9" s="12">
         <v>10</v>
@@ -1647,109 +1690,109 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="21" t="s">
-        <v>12</v>
+      <c r="A10" s="19" t="s">
+        <v>71</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>45</v>
+        <v>16</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>46</v>
+        <v>72</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="E10" s="12">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F10" s="12">
         <v>1.5</v>
       </c>
       <c r="G10" s="12">
-        <v>51.28</v>
+        <v>103.8</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="21" t="s">
-        <v>12</v>
+      <c r="A11" s="19" t="s">
+        <v>71</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>48</v>
+        <v>74</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>49</v>
+        <v>75</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="E11" s="12">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F11" s="12">
         <v>1.57</v>
       </c>
       <c r="G11" s="12">
-        <v>268.37</v>
+        <v>543.24</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="21" t="s">
-        <v>12</v>
+      <c r="A12" s="19" t="s">
+        <v>71</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>51</v>
+        <v>77</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>52</v>
+        <v>78</v>
       </c>
       <c r="E12" s="12">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="F12" s="12">
         <v>0.43</v>
       </c>
       <c r="G12" s="12">
-        <v>44.1</v>
+        <v>89.27</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="21" t="s">
-        <v>12</v>
+      <c r="A13" s="19" t="s">
+        <v>71</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>53</v>
+        <v>79</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>54</v>
+        <v>80</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>55</v>
+        <v>81</v>
       </c>
       <c r="E13" s="12">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F13" s="12">
         <v>1.71</v>
       </c>
       <c r="G13" s="12">
-        <v>58.46</v>
+        <v>118.34</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="21" t="s">
-        <v>12</v>
+      <c r="A14" s="19" t="s">
+        <v>39</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>56</v>
+        <v>82</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>57</v>
+        <v>83</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>58</v>
+        <v>84</v>
       </c>
       <c r="E14" s="12">
         <v>50</v>
@@ -1762,51 +1805,51 @@
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="21" t="s">
-        <v>12</v>
+      <c r="A15" s="19" t="s">
+        <v>71</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>59</v>
+        <v>85</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>60</v>
+        <v>86</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="E15" s="12">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F15" s="12">
         <v>1.61</v>
       </c>
       <c r="G15" s="12">
-        <v>55.04</v>
+        <v>111.41</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>61</v>
+        <v>23</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>62</v>
+        <v>87</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="E16" s="10">
         <v>2</v>
       </c>
-      <c r="F16" s="31">
+      <c r="F16" s="21">
         <f ca="1">77.44*Заказы!L3</f>
-        <v>271.02451200000002</v>
-      </c>
-      <c r="G16" s="31">
+        <v>272.17836799999998</v>
+      </c>
+      <c r="G16" s="21">
         <f ca="1">154.87*Заказы!L3</f>
-        <v>542.01402600000006</v>
+        <v>544.32158900000002</v>
       </c>
     </row>
   </sheetData>
@@ -1829,55 +1872,55 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>65</v>
+        <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>66</v>
+        <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>67</v>
+        <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>68</v>
+        <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>69</v>
+        <v>6</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>70</v>
+        <v>7</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>71</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="25" t="s">
-        <v>72</v>
-      </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
+      <c r="A2" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="6">
         <v>1</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>73</v>
+        <v>11</v>
       </c>
       <c r="D3" s="6">
         <v>95.72</v>
@@ -1905,10 +1948,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>74</v>
+        <v>13</v>
       </c>
       <c r="D4" s="6">
         <v>63.69</v>
@@ -1939,7 +1982,7 @@
         <v>2278432</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>75</v>
+        <v>14</v>
       </c>
       <c r="D5" s="6">
         <v>268.37</v>
@@ -1970,7 +2013,7 @@
         <v>2854115</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>76</v>
+        <v>15</v>
       </c>
       <c r="D6" s="6">
         <v>44.1</v>
@@ -1998,10 +2041,10 @@
         <v>5</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>45</v>
+        <v>16</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>77</v>
+        <v>17</v>
       </c>
       <c r="D7" s="6">
         <v>51.28</v>
@@ -2029,10 +2072,10 @@
         <v>6</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>78</v>
+        <v>19</v>
       </c>
       <c r="D8" s="6">
         <v>592.25</v>
@@ -2055,69 +2098,69 @@
         <v>19.544250000000002</v>
       </c>
       <c r="J8" t="s">
-        <v>85</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="23" t="s">
-        <v>79</v>
-      </c>
-      <c r="B9" s="24"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24"/>
-      <c r="F9" s="24"/>
-      <c r="G9" s="24"/>
-      <c r="H9" s="24"/>
+      <c r="A9" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" s="23"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="23"/>
       <c r="I9" s="4">
         <f>SUM(I3:I8)</f>
         <v>50.390650000000001</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="B10" s="24"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="24"/>
-      <c r="I10" s="24"/>
+      <c r="A10" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="23"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="23"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="10">
         <v>1</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>61</v>
+        <v>23</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>81</v>
+        <v>24</v>
       </c>
       <c r="D11" s="10">
         <f ca="1">154.87*Заказы!L2</f>
-        <v>464.61</v>
+        <v>469.31804800000003</v>
       </c>
       <c r="E11" s="10">
         <v>2</v>
       </c>
       <c r="F11" s="10">
         <f ca="1">IFERROR(D11/E11, 0)</f>
-        <v>232.30500000000001</v>
+        <v>234.65902400000002</v>
       </c>
       <c r="G11" s="10">
         <f ca="1">25.29*Заказы!L2</f>
-        <v>75.87</v>
+        <v>76.638816000000006</v>
       </c>
       <c r="H11" s="10">
         <v>1</v>
       </c>
       <c r="I11" s="10">
         <f ca="1">IFERROR((F11+G11)*H11, 0)</f>
-        <v>308.17500000000001</v>
+        <v>311.29784000000001</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
@@ -2178,35 +2221,35 @@
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" s="23" t="s">
-        <v>82</v>
-      </c>
-      <c r="B15" s="24"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="24"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="24"/>
-      <c r="H15" s="24"/>
+      <c r="A15" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="23"/>
+      <c r="C15" s="23"/>
+      <c r="D15" s="23"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="23"/>
+      <c r="G15" s="23"/>
+      <c r="H15" s="23"/>
       <c r="I15" s="4">
         <f ca="1">SUM(I11:I14)</f>
-        <v>308.17500000000001</v>
+        <v>311.29784000000001</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="26" t="s">
-        <v>83</v>
-      </c>
-      <c r="B16" s="27"/>
-      <c r="C16" s="27"/>
-      <c r="D16" s="27"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="27"/>
-      <c r="G16" s="27"/>
-      <c r="H16" s="28"/>
+      <c r="A16" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="26"/>
+      <c r="C16" s="26"/>
+      <c r="D16" s="26"/>
+      <c r="E16" s="26"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="26"/>
+      <c r="H16" s="27"/>
       <c r="I16" s="9">
         <f ca="1">I9+I15</f>
-        <v>358.56565000000001</v>
+        <v>361.68849</v>
       </c>
     </row>
   </sheetData>
@@ -2229,50 +2272,52 @@
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
     <col min="3" max="3" width="40" customWidth="1"/>
-    <col min="4" max="9" width="15" customWidth="1"/>
+    <col min="4" max="7" width="15" customWidth="1"/>
+    <col min="8" max="8" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>65</v>
+        <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>66</v>
+        <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>67</v>
+        <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>68</v>
+        <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>69</v>
+        <v>6</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>70</v>
+        <v>7</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>71</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="25" t="s">
-        <v>72</v>
-      </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
+      <c r="A2" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
@@ -2351,33 +2396,33 @@
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="23" t="s">
-        <v>79</v>
-      </c>
-      <c r="B7" s="24"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="24"/>
-      <c r="H7" s="24"/>
+      <c r="A7" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="23"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
       <c r="I7" s="4">
         <f>SUM(I3:I6)</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="B8" s="24"/>
-      <c r="C8" s="24"/>
-      <c r="D8" s="24"/>
-      <c r="E8" s="24"/>
-      <c r="F8" s="24"/>
-      <c r="G8" s="24"/>
-      <c r="H8" s="24"/>
-      <c r="I8" s="24"/>
+      <c r="A8" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="23"/>
+      <c r="I8" s="23"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
@@ -2456,32 +2501,32 @@
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="23" t="s">
-        <v>82</v>
-      </c>
-      <c r="B13" s="24"/>
-      <c r="C13" s="24"/>
-      <c r="D13" s="24"/>
-      <c r="E13" s="24"/>
-      <c r="F13" s="24"/>
-      <c r="G13" s="24"/>
-      <c r="H13" s="24"/>
+      <c r="A13" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" s="23"/>
+      <c r="C13" s="23"/>
+      <c r="D13" s="23"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="23"/>
+      <c r="H13" s="23"/>
       <c r="I13" s="4">
         <f>SUM(I9:I12)</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="30" t="s">
-        <v>83</v>
-      </c>
-      <c r="B14" s="24"/>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="24"/>
-      <c r="F14" s="24"/>
-      <c r="G14" s="24"/>
-      <c r="H14" s="24"/>
+      <c r="A14" s="28" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="23"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="23"/>
+      <c r="H14" s="23"/>
       <c r="I14" s="5">
         <f>I7+I13</f>
         <v>0</v>
@@ -2507,50 +2552,52 @@
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
     <col min="3" max="3" width="40" customWidth="1"/>
-    <col min="4" max="9" width="15" customWidth="1"/>
+    <col min="4" max="7" width="15" customWidth="1"/>
+    <col min="8" max="8" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>65</v>
+        <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>66</v>
+        <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>67</v>
+        <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>68</v>
+        <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>69</v>
+        <v>6</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>70</v>
+        <v>7</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>71</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="25" t="s">
-        <v>72</v>
-      </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
+      <c r="A2" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
@@ -2629,33 +2676,33 @@
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="23" t="s">
-        <v>79</v>
-      </c>
-      <c r="B7" s="24"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="24"/>
-      <c r="H7" s="24"/>
+      <c r="A7" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="23"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
       <c r="I7" s="4">
         <f>SUM(I3:I6)</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="B8" s="24"/>
-      <c r="C8" s="24"/>
-      <c r="D8" s="24"/>
-      <c r="E8" s="24"/>
-      <c r="F8" s="24"/>
-      <c r="G8" s="24"/>
-      <c r="H8" s="24"/>
-      <c r="I8" s="24"/>
+      <c r="A8" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="23"/>
+      <c r="I8" s="23"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
@@ -2734,32 +2781,32 @@
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="23" t="s">
-        <v>82</v>
-      </c>
-      <c r="B13" s="24"/>
-      <c r="C13" s="24"/>
-      <c r="D13" s="24"/>
-      <c r="E13" s="24"/>
-      <c r="F13" s="24"/>
-      <c r="G13" s="24"/>
-      <c r="H13" s="24"/>
+      <c r="A13" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" s="23"/>
+      <c r="C13" s="23"/>
+      <c r="D13" s="23"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="23"/>
+      <c r="H13" s="23"/>
       <c r="I13" s="4">
         <f>SUM(I9:I12)</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="30" t="s">
-        <v>83</v>
-      </c>
-      <c r="B14" s="24"/>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="24"/>
-      <c r="F14" s="24"/>
-      <c r="G14" s="24"/>
-      <c r="H14" s="24"/>
+      <c r="A14" s="28" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="23"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="23"/>
+      <c r="H14" s="23"/>
       <c r="I14" s="5">
         <f>I7+I13</f>
         <v>0</v>

</xml_diff>

<commit_message>
PLC RTC and header clock; pressure to displays via room frames; display-to-room binding (config format 2); 'not used' channel option
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Docs/Project_Costs.xlsx
+++ b/Docs/Project_Costs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\morfe\STM32CubeIDE\workspace_1.17.0\HVAC_CleanRoom_Project\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1709863-7257-4908-813E-EAFA5EFF8D15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C871230-6E52-4764-BA49-D31B377DF265}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Заказы" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,8 @@
     <sheet name="Modul_AI" sheetId="3" r:id="rId3"/>
     <sheet name="Modul_Lokomotiv" sheetId="4" r:id="rId4"/>
     <sheet name="Modul_HUB_Displays" sheetId="5" r:id="rId5"/>
+    <sheet name="Modul_Main_PLC" sheetId="6" r:id="rId6"/>
+    <sheet name="Modul_Display" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -84,7 +86,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="122">
   <si>
     <t>№</t>
   </si>
@@ -351,16 +353,118 @@
   </si>
   <si>
     <t>Печатная плата в сборе</t>
+  </si>
+  <si>
+    <t>BC 107,6 UT HBUS BK - Нижняя часть корпуса</t>
+  </si>
+  <si>
+    <t>BC 107,6 OT U22 KMGY - Верхняя часть корпуса</t>
+  </si>
+  <si>
+    <t>BC 53,6 BS U22 KMGY - Заглушка</t>
+  </si>
+  <si>
+    <t>BC 107,6 DKL S TRANS - Крышка корпуса</t>
+  </si>
+  <si>
+    <t>HBUS 107,6-16P-1S BK - Шинный соединитель для установки на монтажную рейку</t>
+  </si>
+  <si>
+    <t>BC 17,6 BS U22 KMGY - Заглушка</t>
+  </si>
+  <si>
+    <t>Сумма, Шек</t>
+  </si>
+  <si>
+    <t>Цена партии, Шек</t>
+  </si>
+  <si>
+    <t>Цена за ед.Шек</t>
+  </si>
+  <si>
+    <t>Цена партии, $</t>
+  </si>
+  <si>
+    <t>Цена за ед.$</t>
+  </si>
+  <si>
+    <t>W2026092620013720</t>
+  </si>
+  <si>
+    <t>Плата часов RTC</t>
+  </si>
+  <si>
+    <t>W2026092617361097</t>
+  </si>
+  <si>
+    <t>Печатная плата Modul_Main_PLC</t>
+  </si>
+  <si>
+    <t>Налоги,Шек</t>
+  </si>
+  <si>
+    <t>Доставка,$</t>
+  </si>
+  <si>
+    <t>Плата CAN_With MINIPower</t>
+  </si>
+  <si>
+    <t>W2026092617531478</t>
+  </si>
+  <si>
+    <t>Плата CAN</t>
+  </si>
+  <si>
+    <t>W2026092022272339</t>
+  </si>
+  <si>
+    <t>W2026092021060492</t>
+  </si>
+  <si>
+    <t>W2026092021170698</t>
+  </si>
+  <si>
+    <t>Печатная плата в сборе Modul_Lokomotiv</t>
+  </si>
+  <si>
+    <t>W2026083101061515</t>
+  </si>
+  <si>
+    <t>Печатная плата в сборе Modul_HUB_Display</t>
+  </si>
+  <si>
+    <t>Верхняя крышка басис на 3D принтере</t>
+  </si>
+  <si>
+    <t>Верхняя крышка лицевая на 3D принтере</t>
+  </si>
+  <si>
+    <t>Задняя крышка на 3D принтере</t>
+  </si>
+  <si>
+    <t>BC 35,6 UT HBUS BK - Нижняя часть корпуса</t>
+  </si>
+  <si>
+    <t>BC 35,6 OT U22 KMGY - Верхняя часть корпуса</t>
+  </si>
+  <si>
+    <t>BC 35,6 DKL S TRANS - Крышка корпуса</t>
+  </si>
+  <si>
+    <t>HBUS 35,6-16P-1S BK - Шинный соединитель для установки на монтажную рейку</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="_ [$₪-40D]\ * #,##0.00_ ;_ [$₪-40D]\ * \-#,##0.00_ ;_ [$₪-40D]\ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="175" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    <numFmt numFmtId="176" formatCode="[$$-409]#,##0.00"/>
+    <numFmt numFmtId="179" formatCode="_ [$₪-40D]\ * #,##0.0000_ ;_ [$₪-40D]\ * \-#,##0.0000_ ;_ [$₪-40D]\ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -417,8 +521,21 @@
       <charset val="204"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF202020"/>
+      <name val="Source Sans Pro"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -473,8 +590,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor rgb="FFE7E6E6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -564,11 +687,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -577,8 +709,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -586,9 +716,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
@@ -609,9 +736,6 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="7" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -627,25 +751,6 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -658,12 +763,82 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="7" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFDDDD09"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -792,17 +967,20 @@
     <v>3</v>
     <v>Finance</v>
     <v>4</v>
-    <v>3.3700999999999999</v>
+    <v>3.3374000000000001</v>
     <v>2.7978000000000001</v>
-    <v>-1.72E-2</v>
-    <v>-5.6439999999999997E-3</v>
+    <v>1.72E-2</v>
+    <v>5.6210000000000001E-3</v>
     <v>ILS</v>
     <v>USD</v>
+    <v>3.0829</v>
     <v>Currency Pair</v>
-    <v>46276.873796296299</v>
+    <v>46307.717372685183</v>
+    <v>3.0617000000000001</v>
     <v>US Dollar/Israeli Shekel FX Spot Rate</v>
-    <v>3.0476000000000001</v>
-    <v>3.0304000000000002</v>
+    <v>3.0668000000000002</v>
+    <v>3.0600999999999998</v>
+    <v>3.0773000000000001</v>
     <v>USDILS</v>
     <v>USD/ILS</v>
   </rv>
@@ -821,17 +999,20 @@
     <v>3</v>
     <v>Finance</v>
     <v>4</v>
-    <v>3.9706999999999999</v>
+    <v>3.8969</v>
     <v>3.2562000000000002</v>
-    <v>-2.3599999999999999E-2</v>
-    <v>-6.6700000000000006E-3</v>
+    <v>6.4000000000000003E-3</v>
+    <v>1.867E-3</v>
     <v>ILS</v>
     <v>EUR</v>
+    <v>3.4506999999999999</v>
     <v>Currency Pair</v>
-    <v>46276.874652777777</v>
+    <v>46307.717372685183</v>
+    <v>3.4264999999999999</v>
     <v>Euro/Israeli Shekel FX Cross Rate</v>
-    <v>3.5383</v>
-    <v>3.5146999999999999</v>
+    <v>3.4264000000000001</v>
+    <v>3.4276</v>
+    <v>3.4340000000000002</v>
     <v>EURILS</v>
     <v>EUR/ILS</v>
   </rv>
@@ -861,9 +1042,12 @@
     <k n="Change (%)"/>
     <k n="Currency" t="s"/>
     <k n="From currency" t="s"/>
+    <k n="High"/>
     <k n="Instrument type" t="s"/>
     <k n="Last trade time"/>
+    <k n="Low"/>
     <k n="Name" t="s"/>
+    <k n="Open"/>
     <k n="Previous close"/>
     <k n="Price"/>
     <k n="Ticker symbol" t="s"/>
@@ -878,7 +1062,7 @@
 <file path=xl/richData/rdsupportingpropertybag.xml><?xml version="1.0" encoding="utf-8"?>
 <supportingPropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2">
   <spbArrays count="1">
-    <a count="24">
+    <a count="27">
       <v t="s">%EntityServiceId</v>
       <v t="s">_Format</v>
       <v t="s">%IsRefreshable</v>
@@ -896,6 +1080,9 @@
       <v t="s">Currency</v>
       <v t="s">From currency</v>
       <v t="s">Previous close</v>
+      <v t="s">Open</v>
+      <v t="s">High</v>
+      <v t="s">Low</v>
       <v t="s">52 week high</v>
       <v t="s">52 week low</v>
       <v t="s">Instrument type</v>
@@ -921,12 +1108,15 @@
     </spb>
     <spb s="3">
       <v>1</v>
+      <v>1</v>
       <v>2</v>
-      <v>2</v>
+      <v>1</v>
+      <v>1</v>
+      <v>1</v>
       <v>3</v>
-      <v>2</v>
-      <v>2</v>
-      <v>2</v>
+      <v>1</v>
+      <v>1</v>
+      <v>1</v>
       <v>4</v>
       <v>5</v>
     </spb>
@@ -953,7 +1143,10 @@
     <k n="`%ProviderInfo" t="spb"/>
   </s>
   <s>
+    <k n="Low" t="i"/>
+    <k n="High" t="i"/>
     <k n="Name" t="i"/>
+    <k n="Open" t="i"/>
     <k n="Price" t="i"/>
     <k n="Change" t="i"/>
     <k n="Change (%)" t="i"/>
@@ -986,20 +1179,20 @@
     </x:dxf>
   </dxfs>
   <richProperties>
+    <rPr n="NumberFormat" t="s"/>
     <rPr n="IsTitleField" t="b"/>
-    <rPr n="NumberFormat" t="s"/>
   </richProperties>
   <richStyles>
+    <rSty dxfid="0">
+      <rpv i="0" xml:space="preserve">_ [$₪-he-IL] * #,##0.00_ ;_ [$₪-he-IL] * -#,##0.00_ ;_ [$₪-he-IL] * "-"??_ ;_ @_ </rpv>
+    </rSty>
     <rSty>
-      <rpv i="0">1</rpv>
-    </rSty>
-    <rSty dxfid="0">
-      <rpv i="1" xml:space="preserve">_ [$₪-he-IL] * #,##0.00_ ;_ [$₪-he-IL] * -#,##0.00_ ;_ [$₪-he-IL] * "-"??_ ;_ @_ </rpv>
+      <rpv i="1">1</rpv>
     </rSty>
     <rSty dxfid="1"/>
     <rSty dxfid="2"/>
     <rSty dxfid="3">
-      <rpv i="1">0.00</rpv>
+      <rpv i="0">0.00</rpv>
     </rSty>
   </richStyles>
 </richStyleSheet>
@@ -1293,14 +1486,14 @@
   <dimension ref="A1:L5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15" style="13" customWidth="1"/>
-    <col min="2" max="2" width="13" style="13" customWidth="1"/>
-    <col min="3" max="3" width="18" style="33" customWidth="1"/>
-    <col min="4" max="4" width="22" style="33" customWidth="1"/>
-    <col min="5" max="5" width="12" style="33" customWidth="1"/>
-    <col min="6" max="6" width="20" style="33" customWidth="1"/>
-    <col min="7" max="7" width="17" style="33" customWidth="1"/>
-    <col min="8" max="8" width="19" style="33" customWidth="1"/>
+    <col min="1" max="1" width="15" style="10" customWidth="1"/>
+    <col min="2" max="2" width="13" style="10" customWidth="1"/>
+    <col min="3" max="3" width="18" style="20" customWidth="1"/>
+    <col min="4" max="4" width="22" style="20" customWidth="1"/>
+    <col min="5" max="5" width="12" style="20" customWidth="1"/>
+    <col min="6" max="6" width="20" style="20" customWidth="1"/>
+    <col min="7" max="7" width="17" style="20" customWidth="1"/>
+    <col min="8" max="8" width="19" style="20" customWidth="1"/>
     <col min="11" max="11" width="13.33203125" customWidth="1"/>
     <col min="12" max="12" width="14.21875" customWidth="1"/>
   </cols>
@@ -1330,129 +1523,129 @@
       <c r="H1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="K1" s="29" t="s">
+      <c r="K1" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="L1" s="30"/>
+      <c r="L1" s="26"/>
     </row>
     <row r="2" spans="1:12" ht="21" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="C2" s="32" t="s">
+      <c r="C2" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="D2" s="34">
+      <c r="D2" s="21">
         <v>1815.8</v>
       </c>
-      <c r="E2" s="34">
+      <c r="E2" s="21">
         <v>326.83999999999997</v>
       </c>
-      <c r="F2" s="34">
+      <c r="F2" s="21">
         <v>2142.64</v>
       </c>
-      <c r="G2" s="34">
-        <v>0</v>
-      </c>
-      <c r="H2" s="34">
-        <v>0</v>
-      </c>
-      <c r="K2" s="15" t="e" vm="1">
+      <c r="G2" s="21">
+        <v>0</v>
+      </c>
+      <c r="H2" s="21">
+        <v>0</v>
+      </c>
+      <c r="K2" s="12" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="L2" s="16" cm="1">
+      <c r="L2" s="38" cm="1">
         <f t="array" aca="1" ref="L2" ca="1">_FV(K2,"Price")</f>
-        <v>3.0304000000000002</v>
+        <v>3.0773000000000001</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="32" t="s">
+      <c r="C3" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="D3" s="34">
+      <c r="D3" s="21">
         <v>825.96</v>
       </c>
-      <c r="E3" s="34">
+      <c r="E3" s="21">
         <v>148.66999999999999</v>
       </c>
-      <c r="F3" s="34">
+      <c r="F3" s="21">
         <v>974.63</v>
       </c>
-      <c r="G3" s="34">
-        <v>0</v>
-      </c>
-      <c r="H3" s="34">
-        <v>0</v>
-      </c>
-      <c r="K3" s="15" t="e" vm="2">
+      <c r="G3" s="21">
+        <v>0</v>
+      </c>
+      <c r="H3" s="21">
+        <v>0</v>
+      </c>
+      <c r="K3" s="12" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="L3" s="17" cm="1">
+      <c r="L3" s="13" cm="1">
         <f t="array" aca="1" ref="L3" ca="1">_FV(K3,"Price")</f>
-        <v>3.5146999999999999</v>
+        <v>3.4340000000000002</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="D4" s="18">
+      <c r="D4" s="14">
         <f ca="1">156.07*L2</f>
-        <v>472.95452800000004</v>
-      </c>
-      <c r="E4" s="18">
-        <v>0</v>
-      </c>
-      <c r="F4" s="18">
+        <v>480.27421099999998</v>
+      </c>
+      <c r="E4" s="14">
+        <v>0</v>
+      </c>
+      <c r="F4" s="14">
         <f ca="1">156.07*L2</f>
-        <v>472.95452800000004</v>
-      </c>
-      <c r="G4" s="18">
+        <v>480.27421099999998</v>
+      </c>
+      <c r="G4" s="14">
         <f ca="1">25.29*L2</f>
-        <v>76.638816000000006</v>
-      </c>
-      <c r="H4" s="18">
+        <v>77.824916999999999</v>
+      </c>
+      <c r="H4" s="14">
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A5" s="31" t="s">
+      <c r="A5" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="31" t="s">
+      <c r="B5" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="31" t="s">
+      <c r="C5" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="D5" s="18">
+      <c r="D5" s="14">
         <v>488.98</v>
       </c>
-      <c r="E5" s="18">
+      <c r="E5" s="14">
         <v>88.02</v>
       </c>
-      <c r="F5" s="18">
+      <c r="F5" s="14">
         <v>577</v>
       </c>
-      <c r="G5" s="18">
-        <v>0</v>
-      </c>
-      <c r="H5" s="18">
+      <c r="G5" s="14">
+        <v>0</v>
+      </c>
+      <c r="H5" s="14">
         <v>0</v>
       </c>
       <c r="K5">
@@ -1473,17 +1666,17 @@
   <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.21875" style="20" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.21875" style="16" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="40.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="32.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.109375" style="13" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.44140625" style="13" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.44140625" style="13" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.109375" style="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.44140625" style="10" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.44140625" style="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="11" t="s">
         <v>27</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -1506,7 +1699,7 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="15" t="s">
         <v>36</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -1518,18 +1711,18 @@
       <c r="D2" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E2" s="12">
+      <c r="E2" s="9">
         <v>10</v>
       </c>
-      <c r="F2" s="12">
+      <c r="F2" s="9">
         <v>2.72</v>
       </c>
-      <c r="G2" s="12">
+      <c r="G2" s="9">
         <v>95.72</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="15" t="s">
         <v>36</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -1541,18 +1734,18 @@
       <c r="D3" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="9">
         <v>10</v>
       </c>
-      <c r="F3" s="12">
+      <c r="F3" s="9">
         <v>1.22</v>
       </c>
-      <c r="G3" s="12">
+      <c r="G3" s="9">
         <v>42.93</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="15" t="s">
         <v>36</v>
       </c>
       <c r="B4" s="2" t="s">
@@ -1564,18 +1757,18 @@
       <c r="D4" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E4" s="12">
+      <c r="E4" s="9">
         <v>10</v>
       </c>
-      <c r="F4" s="12">
+      <c r="F4" s="9">
         <v>16.829999999999998</v>
       </c>
-      <c r="G4" s="12">
+      <c r="G4" s="9">
         <v>592.25</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="15" t="s">
         <v>36</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -1587,18 +1780,18 @@
       <c r="D5" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E5" s="12">
+      <c r="E5" s="9">
         <v>50</v>
       </c>
-      <c r="F5" s="12">
+      <c r="F5" s="9">
         <v>1.94</v>
       </c>
-      <c r="G5" s="12">
+      <c r="G5" s="9">
         <v>341.34</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="15" t="s">
         <v>36</v>
       </c>
       <c r="B6" s="2" t="s">
@@ -1610,18 +1803,18 @@
       <c r="D6" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="E6" s="12">
+      <c r="E6" s="9">
         <v>50</v>
       </c>
-      <c r="F6" s="12">
+      <c r="F6" s="9">
         <v>0.56000000000000005</v>
       </c>
-      <c r="G6" s="12">
+      <c r="G6" s="9">
         <v>98.53</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="15" t="s">
         <v>36</v>
       </c>
       <c r="B7" s="2" t="s">
@@ -1633,18 +1826,18 @@
       <c r="D7" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="E7" s="12">
+      <c r="E7" s="9">
         <v>50</v>
       </c>
-      <c r="F7" s="12">
+      <c r="F7" s="9">
         <v>1.0900000000000001</v>
       </c>
-      <c r="G7" s="12">
+      <c r="G7" s="9">
         <v>191.79</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="15" t="s">
         <v>36</v>
       </c>
       <c r="B8" s="2" t="s">
@@ -1656,18 +1849,18 @@
       <c r="D8" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E8" s="12">
+      <c r="E8" s="9">
         <v>10</v>
       </c>
-      <c r="F8" s="12">
+      <c r="F8" s="9">
         <v>1.81</v>
       </c>
-      <c r="G8" s="12">
+      <c r="G8" s="9">
         <v>63.69</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="15" t="s">
         <v>36</v>
       </c>
       <c r="B9" s="2" t="s">
@@ -1679,18 +1872,18 @@
       <c r="D9" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E9" s="12">
+      <c r="E9" s="9">
         <v>10</v>
       </c>
-      <c r="F9" s="12">
+      <c r="F9" s="9">
         <v>11.07</v>
       </c>
-      <c r="G9" s="12">
+      <c r="G9" s="9">
         <v>389.55</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="15" t="s">
         <v>71</v>
       </c>
       <c r="B10" s="2" t="s">
@@ -1702,18 +1895,18 @@
       <c r="D10" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="9">
         <v>20</v>
       </c>
-      <c r="F10" s="12">
+      <c r="F10" s="9">
         <v>1.5</v>
       </c>
-      <c r="G10" s="12">
+      <c r="G10" s="9">
         <v>103.8</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="15" t="s">
         <v>71</v>
       </c>
       <c r="B11" s="2" t="s">
@@ -1725,18 +1918,18 @@
       <c r="D11" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E11" s="12">
+      <c r="E11" s="9">
         <v>100</v>
       </c>
-      <c r="F11" s="12">
+      <c r="F11" s="9">
         <v>1.57</v>
       </c>
-      <c r="G11" s="12">
+      <c r="G11" s="9">
         <v>543.24</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="15" t="s">
         <v>71</v>
       </c>
       <c r="B12" s="2" t="s">
@@ -1748,18 +1941,18 @@
       <c r="D12" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E12" s="12">
+      <c r="E12" s="9">
         <v>60</v>
       </c>
-      <c r="F12" s="12">
+      <c r="F12" s="9">
         <v>0.43</v>
       </c>
-      <c r="G12" s="12">
+      <c r="G12" s="9">
         <v>89.27</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="15" t="s">
         <v>71</v>
       </c>
       <c r="B13" s="2" t="s">
@@ -1771,18 +1964,18 @@
       <c r="D13" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="E13" s="12">
+      <c r="E13" s="9">
         <v>20</v>
       </c>
-      <c r="F13" s="12">
+      <c r="F13" s="9">
         <v>1.71</v>
       </c>
-      <c r="G13" s="12">
+      <c r="G13" s="9">
         <v>118.34</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="19" t="s">
+      <c r="A14" s="15" t="s">
         <v>39</v>
       </c>
       <c r="B14" s="2" t="s">
@@ -1794,18 +1987,18 @@
       <c r="D14" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="E14" s="12">
+      <c r="E14" s="9">
         <v>50</v>
       </c>
-      <c r="F14" s="12">
+      <c r="F14" s="9">
         <v>2.04</v>
       </c>
-      <c r="G14" s="12">
+      <c r="G14" s="9">
         <v>348.71</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="15" t="s">
         <v>71</v>
       </c>
       <c r="B15" s="2" t="s">
@@ -1817,39 +2010,39 @@
       <c r="D15" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E15" s="12">
+      <c r="E15" s="9">
         <v>20</v>
       </c>
-      <c r="F15" s="12">
+      <c r="F15" s="9">
         <v>1.61</v>
       </c>
-      <c r="G15" s="12">
+      <c r="G15" s="9">
         <v>111.41</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="C16" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="E16" s="10">
+      <c r="E16" s="7">
         <v>2</v>
       </c>
-      <c r="F16" s="21">
+      <c r="F16" s="17">
         <f ca="1">77.44*Заказы!L3</f>
-        <v>272.17836799999998</v>
-      </c>
-      <c r="G16" s="21">
+        <v>265.92896000000002</v>
+      </c>
+      <c r="G16" s="17">
         <f ca="1">154.87*Заказы!L3</f>
-        <v>544.32158900000002</v>
+        <v>531.82357999999999</v>
       </c>
     </row>
   </sheetData>
@@ -1859,15 +2052,19 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="1" max="1" width="3.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="51.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="15" customWidth="1"/>
-    <col min="8" max="8" width="21.33203125" customWidth="1"/>
-    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="4" max="4" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
@@ -1913,187 +2110,187 @@
       <c r="I2" s="23"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="6">
-        <v>1</v>
-      </c>
-      <c r="B3" s="6" t="s">
+      <c r="A3" s="4">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="6">
-        <v>95.72</v>
-      </c>
-      <c r="E3" s="6">
+      <c r="D3" s="30">
+        <v>122.42</v>
+      </c>
+      <c r="E3" s="4">
         <v>10</v>
       </c>
-      <c r="F3" s="6">
-        <f t="shared" ref="F3:F8" si="0">IFERROR(D3/E3, 0)</f>
-        <v>9.5719999999999992</v>
-      </c>
-      <c r="G3" s="6">
-        <v>0</v>
-      </c>
-      <c r="H3" s="6">
-        <v>1</v>
-      </c>
-      <c r="I3" s="6">
-        <f t="shared" ref="I3:I8" si="1">IFERROR((F3+G3)*H3, 0)</f>
-        <v>9.5719999999999992</v>
+      <c r="F3" s="30">
+        <f>SUM(D3/E3)</f>
+        <v>12.242000000000001</v>
+      </c>
+      <c r="G3" s="30">
+        <v>0</v>
+      </c>
+      <c r="H3" s="4">
+        <v>1</v>
+      </c>
+      <c r="I3" s="30">
+        <f>SUM(F3*H3+G3/E3)</f>
+        <v>12.242000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="6">
+      <c r="A4" s="4">
         <v>2</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="30">
         <v>63.69</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="4">
         <v>10</v>
       </c>
-      <c r="F4" s="6">
-        <f t="shared" si="0"/>
+      <c r="F4" s="30">
+        <f t="shared" ref="F4:F8" si="0">SUM(D4/E4)</f>
         <v>6.3689999999999998</v>
       </c>
-      <c r="G4" s="6">
-        <v>0</v>
-      </c>
-      <c r="H4" s="6">
-        <v>1</v>
-      </c>
-      <c r="I4" s="6">
-        <f t="shared" si="1"/>
+      <c r="G4" s="30">
+        <v>0</v>
+      </c>
+      <c r="H4" s="4">
+        <v>1</v>
+      </c>
+      <c r="I4" s="30">
+        <f t="shared" ref="I4:I8" si="1">SUM(F4*H4+G4/E4)</f>
         <v>6.3689999999999998</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="6">
+      <c r="A5" s="4">
         <v>3</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="6">
         <v>2278432</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="30">
         <v>268.37</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="4">
         <v>50</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="30">
         <f t="shared" si="0"/>
         <v>5.3673999999999999</v>
       </c>
-      <c r="G5" s="6">
-        <v>0</v>
-      </c>
-      <c r="H5" s="6">
-        <v>1</v>
-      </c>
-      <c r="I5" s="6">
+      <c r="G5" s="30">
+        <v>0</v>
+      </c>
+      <c r="H5" s="4">
+        <v>1</v>
+      </c>
+      <c r="I5" s="30">
         <f t="shared" si="1"/>
         <v>5.3673999999999999</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="6">
+      <c r="A6" s="4">
         <v>4</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="6">
         <v>2854115</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="30">
         <v>44.1</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="4">
         <v>30</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="30">
         <f t="shared" si="0"/>
         <v>1.47</v>
       </c>
-      <c r="G6" s="6">
-        <v>0</v>
-      </c>
-      <c r="H6" s="6">
+      <c r="G6" s="30">
+        <v>0</v>
+      </c>
+      <c r="H6" s="4">
         <v>3</v>
       </c>
-      <c r="I6" s="6">
+      <c r="I6" s="30">
         <f t="shared" si="1"/>
         <v>4.41</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="6">
+      <c r="A7" s="4">
         <v>5</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="30">
         <v>51.28</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="4">
         <v>10</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="30">
         <f t="shared" si="0"/>
         <v>5.1280000000000001</v>
       </c>
-      <c r="G7" s="6">
-        <v>0</v>
-      </c>
-      <c r="H7" s="6">
-        <v>1</v>
-      </c>
-      <c r="I7" s="6">
+      <c r="G7" s="30">
+        <v>0</v>
+      </c>
+      <c r="H7" s="4">
+        <v>1</v>
+      </c>
+      <c r="I7" s="30">
         <f t="shared" si="1"/>
         <v>5.1280000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="6">
+      <c r="A8" s="4">
         <v>6</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="30">
         <v>592.25</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="4">
         <v>10</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="30">
         <f t="shared" si="0"/>
         <v>59.225000000000001</v>
       </c>
-      <c r="G8" s="6">
-        <v>0</v>
-      </c>
-      <c r="H8" s="6">
+      <c r="G8" s="30">
+        <v>0</v>
+      </c>
+      <c r="H8" s="4">
         <v>0.33</v>
       </c>
-      <c r="I8" s="6">
+      <c r="I8" s="30">
         <f t="shared" si="1"/>
         <v>19.544250000000002</v>
       </c>
@@ -2112,153 +2309,132 @@
       <c r="F9" s="23"/>
       <c r="G9" s="23"/>
       <c r="H9" s="23"/>
-      <c r="I9" s="4">
+      <c r="I9" s="39">
         <f>SUM(I3:I8)</f>
-        <v>50.390650000000001</v>
+        <v>53.06065000000001</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="24" t="s">
+      <c r="A10" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="23"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="23"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="23"/>
-      <c r="G10" s="23"/>
-      <c r="H10" s="23"/>
-      <c r="I10" s="23"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="10">
-        <v>1</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" s="11" t="s">
+      <c r="B10" s="42"/>
+      <c r="C10" s="42"/>
+      <c r="D10" s="42"/>
+      <c r="E10" s="42"/>
+      <c r="F10" s="42"/>
+      <c r="G10" s="42"/>
+      <c r="H10" s="42"/>
+      <c r="I10" s="42"/>
+      <c r="J10" s="42"/>
+    </row>
+    <row r="11" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D11" s="29" t="s">
+        <v>98</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F11" s="29" t="s">
+        <v>99</v>
+      </c>
+      <c r="G11" s="29" t="s">
+        <v>105</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I11" s="35" t="s">
+        <v>104</v>
+      </c>
+      <c r="J11" s="29" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" s="7">
+        <v>1</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C12" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="10">
-        <f ca="1">154.87*Заказы!L2</f>
-        <v>469.31804800000003</v>
-      </c>
-      <c r="E11" s="10">
-        <v>2</v>
-      </c>
-      <c r="F11" s="10">
-        <f ca="1">IFERROR(D11/E11, 0)</f>
-        <v>234.65902400000002</v>
-      </c>
-      <c r="G11" s="10">
-        <f ca="1">25.29*Заказы!L2</f>
-        <v>76.638816000000006</v>
-      </c>
-      <c r="H11" s="10">
-        <v>1</v>
-      </c>
-      <c r="I11" s="10">
-        <f ca="1">IFERROR((F11+G11)*H11, 0)</f>
-        <v>311.29784000000001</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="6">
-        <v>2</v>
-      </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6">
-        <f>IFERROR(D12/E12, 0)</f>
-        <v>0</v>
-      </c>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6">
-        <f>IFERROR((F12+G12)*H12, 0)</f>
-        <v>0</v>
+      <c r="D12" s="7">
+        <v>301.95</v>
+      </c>
+      <c r="E12" s="7">
+        <v>10</v>
+      </c>
+      <c r="F12" s="41">
+        <f>SUM(D12/E12)</f>
+        <v>30.195</v>
+      </c>
+      <c r="G12" s="7">
+        <v>28.14</v>
+      </c>
+      <c r="H12" s="7">
+        <v>1</v>
+      </c>
+      <c r="I12" s="7">
+        <v>414</v>
+      </c>
+      <c r="J12" s="14">
+        <f ca="1">(F12+G12/E12)*Заказы!$L$2+I12/E12</f>
+        <v>142.9785957</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="6">
-        <v>3</v>
-      </c>
-      <c r="B13" s="6"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6">
-        <f>IFERROR(D13/E13, 0)</f>
-        <v>0</v>
-      </c>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6">
-        <f>IFERROR((F13+G13)*H13, 0)</f>
-        <v>0</v>
+      <c r="A13" s="32" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" s="32"/>
+      <c r="C13" s="32"/>
+      <c r="D13" s="32"/>
+      <c r="E13" s="32"/>
+      <c r="F13" s="32"/>
+      <c r="G13" s="32"/>
+      <c r="H13" s="32"/>
+      <c r="I13" s="33"/>
+      <c r="J13" s="39">
+        <f ca="1">SUM(J12)</f>
+        <v>142.9785957</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="6">
-        <v>4</v>
-      </c>
-      <c r="B14" s="6"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6">
-        <f>IFERROR(D14/E14, 0)</f>
-        <v>0</v>
-      </c>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="6">
-        <f>IFERROR((F14+G14)*H14, 0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B15" s="23"/>
-      <c r="C15" s="23"/>
-      <c r="D15" s="23"/>
-      <c r="E15" s="23"/>
-      <c r="F15" s="23"/>
-      <c r="G15" s="23"/>
-      <c r="H15" s="23"/>
-      <c r="I15" s="4">
-        <f ca="1">SUM(I11:I14)</f>
-        <v>311.29784000000001</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="25" t="s">
+      <c r="A14" s="43" t="s">
         <v>26</v>
       </c>
-      <c r="B16" s="26"/>
-      <c r="C16" s="26"/>
-      <c r="D16" s="26"/>
-      <c r="E16" s="26"/>
-      <c r="F16" s="26"/>
-      <c r="G16" s="26"/>
-      <c r="H16" s="27"/>
-      <c r="I16" s="9">
-        <f ca="1">I9+I15</f>
-        <v>361.68849</v>
+      <c r="B14" s="44"/>
+      <c r="C14" s="44"/>
+      <c r="D14" s="44"/>
+      <c r="E14" s="44"/>
+      <c r="F14" s="44"/>
+      <c r="G14" s="44"/>
+      <c r="H14" s="44"/>
+      <c r="I14" s="45"/>
+      <c r="J14" s="46">
+        <f ca="1">J13+I9</f>
+        <v>196.03924570000001</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A9:H9"/>
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A15:H15"/>
-    <mergeCell ref="A10:I10"/>
-    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A10:J10"/>
+    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="A14:I14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2266,18 +2442,22 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="40" customWidth="1"/>
-    <col min="4" max="7" width="15" customWidth="1"/>
+    <col min="1" max="1" width="3.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="71.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="9" max="9" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -2306,7 +2486,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="24" t="s">
         <v>9</v>
       </c>
@@ -2319,101 +2499,160 @@
       <c r="H2" s="23"/>
       <c r="I2" s="23"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="2">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2">
-        <f>IFERROR(D3/E3, 0)</f>
-        <v>0</v>
-      </c>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2">
-        <f>IFERROR((F3+G3)*H3, 0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="4">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4">
+        <v>2896254</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="D3" s="30"/>
+      <c r="E3" s="4">
+        <v>10</v>
+      </c>
+      <c r="F3" s="30">
+        <f>SUM(D3/E3)</f>
+        <v>0</v>
+      </c>
+      <c r="G3" s="30">
+        <v>0</v>
+      </c>
+      <c r="H3" s="4">
+        <v>1</v>
+      </c>
+      <c r="I3" s="30">
+        <f>SUM(F3*H3+G3/E3)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="4">
         <v>2</v>
       </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2">
-        <f>IFERROR(D4/E4, 0)</f>
-        <v>0</v>
-      </c>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2">
-        <f>IFERROR((F4+G4)*H4, 0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="2">
-        <v>3</v>
-      </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2">
-        <f>IFERROR(D5/E5, 0)</f>
-        <v>0</v>
-      </c>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2">
-        <f>IFERROR((F5+G5)*H5, 0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="2">
+      <c r="B4" s="4">
+        <v>2896047</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="D4" s="30"/>
+      <c r="E4" s="4">
+        <v>10</v>
+      </c>
+      <c r="F4" s="30">
+        <f t="shared" ref="F4:F7" si="0">SUM(D4/E4)</f>
+        <v>0</v>
+      </c>
+      <c r="G4" s="30">
+        <v>0</v>
+      </c>
+      <c r="H4" s="4">
+        <v>1</v>
+      </c>
+      <c r="I4" s="30">
+        <f t="shared" ref="I4:I7" si="1">SUM(F4*H4+G4/E4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="4">
         <v>4</v>
       </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2">
-        <f>IFERROR(D6/E6, 0)</f>
-        <v>0</v>
-      </c>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2">
-        <f>IFERROR((F6+G6)*H6, 0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="22" t="s">
+      <c r="B5" s="6">
+        <v>2896199</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D5" s="30">
+        <v>348.71</v>
+      </c>
+      <c r="E5" s="4">
+        <v>50</v>
+      </c>
+      <c r="F5" s="30">
+        <f t="shared" si="0"/>
+        <v>6.9741999999999997</v>
+      </c>
+      <c r="G5" s="30">
+        <v>0</v>
+      </c>
+      <c r="H5" s="4">
+        <v>1</v>
+      </c>
+      <c r="I5" s="30">
+        <f t="shared" si="1"/>
+        <v>6.9741999999999997</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="4">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4">
+        <v>2896115</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="D6" s="30">
+        <v>55.04</v>
+      </c>
+      <c r="E6" s="4">
+        <v>10</v>
+      </c>
+      <c r="F6" s="30">
+        <f t="shared" si="0"/>
+        <v>5.5039999999999996</v>
+      </c>
+      <c r="G6" s="30">
+        <v>0</v>
+      </c>
+      <c r="H6" s="4">
+        <v>1</v>
+      </c>
+      <c r="I6" s="30">
+        <f t="shared" si="1"/>
+        <v>5.5039999999999996</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="4">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4">
+        <v>2896283</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="D7" s="30">
+        <v>389.55</v>
+      </c>
+      <c r="E7" s="4">
+        <v>10</v>
+      </c>
+      <c r="F7" s="30">
+        <f t="shared" si="0"/>
+        <v>38.954999999999998</v>
+      </c>
+      <c r="G7" s="30">
+        <v>0</v>
+      </c>
+      <c r="H7" s="4">
+        <v>1</v>
+      </c>
+      <c r="I7" s="30">
+        <f t="shared" si="1"/>
+        <v>38.954999999999998</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" s="22" t="s">
         <v>21</v>
-      </c>
-      <c r="B7" s="23"/>
-      <c r="C7" s="23"/>
-      <c r="D7" s="23"/>
-      <c r="E7" s="23"/>
-      <c r="F7" s="23"/>
-      <c r="G7" s="23"/>
-      <c r="H7" s="23"/>
-      <c r="I7" s="4">
-        <f>SUM(I3:I6)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="24" t="s">
-        <v>22</v>
       </c>
       <c r="B8" s="23"/>
       <c r="C8" s="23"/>
@@ -2422,142 +2661,223 @@
       <c r="F8" s="23"/>
       <c r="G8" s="23"/>
       <c r="H8" s="23"/>
-      <c r="I8" s="23"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="2">
-        <v>1</v>
-      </c>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2">
-        <f>IFERROR(D9/E9, 0)</f>
-        <v>0</v>
-      </c>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2">
-        <f>IFERROR((F9+G9)*H9, 0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="2">
+      <c r="I8" s="39">
+        <f>SUM(I3:I7)</f>
+        <v>51.433199999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="42" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="42"/>
+      <c r="C9" s="42"/>
+      <c r="D9" s="42"/>
+      <c r="E9" s="42"/>
+      <c r="F9" s="42"/>
+      <c r="G9" s="42"/>
+      <c r="H9" s="42"/>
+      <c r="I9" s="42"/>
+      <c r="J9" s="42"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2">
-        <f>IFERROR(D10/E10, 0)</f>
-        <v>0</v>
-      </c>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2">
-        <f>IFERROR((F10+G10)*H10, 0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="2">
+      <c r="D10" s="29" t="s">
+        <v>98</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F10" s="29" t="s">
+        <v>99</v>
+      </c>
+      <c r="G10" s="29" t="s">
+        <v>105</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I10" s="35" t="s">
+        <v>104</v>
+      </c>
+      <c r="J10" s="29" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" s="7">
+        <v>1</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="D11" s="37">
+        <v>167.54</v>
+      </c>
+      <c r="E11" s="7">
+        <v>25</v>
+      </c>
+      <c r="F11" s="36">
+        <f>SUM(D11/E11)</f>
+        <v>6.7016</v>
+      </c>
+      <c r="G11" s="36">
+        <v>56.39</v>
+      </c>
+      <c r="H11" s="7">
+        <v>1</v>
+      </c>
+      <c r="I11" s="14">
+        <v>356</v>
+      </c>
+      <c r="J11" s="14">
+        <f ca="1">(F11+G11/E11)*Заказы!$L$2+I11/E11</f>
+        <v>41.80399156</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" s="4">
+        <v>2</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="D12" s="37">
+        <v>274.17</v>
+      </c>
+      <c r="E12" s="7">
+        <v>50</v>
+      </c>
+      <c r="F12" s="36">
+        <f t="shared" ref="F11:F12" si="2">SUM(D12/E12)</f>
+        <v>5.4834000000000005</v>
+      </c>
+      <c r="G12" s="36">
+        <v>43.72</v>
+      </c>
+      <c r="H12" s="7">
+        <v>1</v>
+      </c>
+      <c r="I12" s="14">
+        <v>407</v>
+      </c>
+      <c r="J12" s="14">
+        <f ca="1">(F12+G12/E12)*Заказы!$L$2+I12/E12</f>
+        <v>27.70485794</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13" s="4">
         <v>3</v>
       </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2">
-        <f>IFERROR(D11/E11, 0)</f>
-        <v>0</v>
-      </c>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2">
-        <f>IFERROR((F11+G11)*H11, 0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="2">
-        <v>4</v>
-      </c>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2">
-        <f>IFERROR(D12/E12, 0)</f>
-        <v>0</v>
-      </c>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2">
-        <f>IFERROR((F12+G12)*H12, 0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="22" t="s">
+      <c r="B13" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="D13" s="37">
+        <v>283.99</v>
+      </c>
+      <c r="E13" s="7">
+        <v>50</v>
+      </c>
+      <c r="F13" s="36">
+        <v>56.39</v>
+      </c>
+      <c r="G13" s="36">
+        <v>43.72</v>
+      </c>
+      <c r="H13" s="7">
+        <v>1</v>
+      </c>
+      <c r="I13" s="14">
+        <v>419</v>
+      </c>
+      <c r="J13" s="14">
+        <f ca="1">(F13+G13/E13)*Заказы!$L$2+I13/E13</f>
+        <v>184.59973812000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A14" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="23"/>
-      <c r="C13" s="23"/>
-      <c r="D13" s="23"/>
-      <c r="E13" s="23"/>
-      <c r="F13" s="23"/>
-      <c r="G13" s="23"/>
-      <c r="H13" s="23"/>
-      <c r="I13" s="4">
-        <f>SUM(I9:I12)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="28" t="s">
+      <c r="B14" s="32"/>
+      <c r="C14" s="32"/>
+      <c r="D14" s="32"/>
+      <c r="E14" s="32"/>
+      <c r="F14" s="32"/>
+      <c r="G14" s="32"/>
+      <c r="H14" s="32"/>
+      <c r="I14" s="33"/>
+      <c r="J14" s="39">
+        <f ca="1">SUM(J11:J13)</f>
+        <v>254.10858762000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15" s="43" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="23"/>
-      <c r="C14" s="23"/>
-      <c r="D14" s="23"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="23"/>
-      <c r="H14" s="23"/>
-      <c r="I14" s="5">
-        <f>I7+I13</f>
-        <v>0</v>
+      <c r="B15" s="44"/>
+      <c r="C15" s="44"/>
+      <c r="D15" s="44"/>
+      <c r="E15" s="44"/>
+      <c r="F15" s="44"/>
+      <c r="G15" s="44"/>
+      <c r="H15" s="44"/>
+      <c r="I15" s="45"/>
+      <c r="J15" s="46">
+        <f ca="1">J14+I8</f>
+        <v>305.54178762000004</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A8:I8"/>
-    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="A14:I14"/>
+    <mergeCell ref="A15:I15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="40" customWidth="1"/>
-    <col min="4" max="7" width="15" customWidth="1"/>
+    <col min="1" max="1" width="3.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="72.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="9" max="9" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -2586,7 +2906,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="24" t="s">
         <v>9</v>
       </c>
@@ -2599,101 +2919,144 @@
       <c r="H2" s="23"/>
       <c r="I2" s="23"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="2">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2">
-        <f>IFERROR(D3/E3, 0)</f>
-        <v>0</v>
-      </c>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2">
-        <f>IFERROR((F3+G3)*H3, 0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="4">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4">
+        <v>2896270</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="D3" s="30">
+        <v>122.42</v>
+      </c>
+      <c r="E3" s="4">
+        <v>10</v>
+      </c>
+      <c r="F3" s="30">
+        <f>SUM(D3/E3)</f>
+        <v>12.242000000000001</v>
+      </c>
+      <c r="G3" s="4">
+        <v>0</v>
+      </c>
+      <c r="H3" s="4">
+        <v>1</v>
+      </c>
+      <c r="I3" s="30">
+        <f>SUM(F3*H3+G3)</f>
+        <v>12.242000000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="4">
         <v>2</v>
       </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2">
-        <f>IFERROR(D4/E4, 0)</f>
-        <v>0</v>
-      </c>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2">
-        <f>IFERROR((F4+G4)*H4, 0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="2">
+      <c r="B4" s="4">
+        <v>2896089</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="D4" s="30">
+        <v>91.3</v>
+      </c>
+      <c r="E4" s="4">
+        <v>10</v>
+      </c>
+      <c r="F4" s="30">
+        <f t="shared" ref="F4:F6" si="0">SUM(D4/E4)</f>
+        <v>9.129999999999999</v>
+      </c>
+      <c r="G4" s="4">
+        <v>0</v>
+      </c>
+      <c r="H4" s="4">
+        <v>1</v>
+      </c>
+      <c r="I4" s="30">
+        <f t="shared" ref="I4:I6" si="1">SUM(F4*H4+G4)</f>
+        <v>9.129999999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="4">
         <v>3</v>
       </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2">
-        <f>IFERROR(D5/E5, 0)</f>
-        <v>0</v>
-      </c>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2">
-        <f>IFERROR((F5+G5)*H5, 0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="2">
+      <c r="B5" s="4">
+        <v>2896131</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="D5" s="30">
+        <v>72.62</v>
+      </c>
+      <c r="E5" s="4">
+        <v>10</v>
+      </c>
+      <c r="F5" s="30">
+        <f t="shared" si="0"/>
+        <v>7.2620000000000005</v>
+      </c>
+      <c r="G5" s="4">
+        <v>0</v>
+      </c>
+      <c r="H5" s="4">
+        <v>1</v>
+      </c>
+      <c r="I5" s="30">
+        <f t="shared" si="1"/>
+        <v>7.2620000000000005</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="4">
         <v>4</v>
       </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2">
-        <f>IFERROR(D6/E6, 0)</f>
-        <v>0</v>
-      </c>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2">
-        <f>IFERROR((F6+G6)*H6, 0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="22" t="s">
+      <c r="B6" s="4">
+        <v>2896306</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="D6" s="30">
+        <v>540.88</v>
+      </c>
+      <c r="E6" s="4">
+        <v>10</v>
+      </c>
+      <c r="F6" s="30">
+        <f t="shared" si="0"/>
+        <v>54.088000000000001</v>
+      </c>
+      <c r="G6" s="4">
+        <v>0</v>
+      </c>
+      <c r="H6" s="4">
+        <v>1</v>
+      </c>
+      <c r="I6" s="30">
+        <f t="shared" si="1"/>
+        <v>54.088000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="27"/>
+      <c r="B7" s="27"/>
+      <c r="C7" s="28"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
+      <c r="H7" s="27"/>
+      <c r="I7" s="7"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" s="22" t="s">
         <v>21</v>
-      </c>
-      <c r="B7" s="23"/>
-      <c r="C7" s="23"/>
-      <c r="D7" s="23"/>
-      <c r="E7" s="23"/>
-      <c r="F7" s="23"/>
-      <c r="G7" s="23"/>
-      <c r="H7" s="23"/>
-      <c r="I7" s="4">
-        <f>SUM(I3:I6)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="24" t="s">
-        <v>22</v>
       </c>
       <c r="B8" s="23"/>
       <c r="C8" s="23"/>
@@ -2702,124 +3065,987 @@
       <c r="F8" s="23"/>
       <c r="G8" s="23"/>
       <c r="H8" s="23"/>
-      <c r="I8" s="23"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="2">
-        <v>1</v>
-      </c>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2">
-        <f>IFERROR(D9/E9, 0)</f>
-        <v>0</v>
-      </c>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2">
-        <f>IFERROR((F9+G9)*H9, 0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="2">
+      <c r="I8" s="39">
+        <f>SUM(I3:I7)</f>
+        <v>82.722000000000008</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="42" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="42"/>
+      <c r="C9" s="42"/>
+      <c r="D9" s="42"/>
+      <c r="E9" s="42"/>
+      <c r="F9" s="42"/>
+      <c r="G9" s="42"/>
+      <c r="H9" s="42"/>
+      <c r="I9" s="42"/>
+      <c r="J9" s="42"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2">
-        <f>IFERROR(D10/E10, 0)</f>
-        <v>0</v>
-      </c>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2">
-        <f>IFERROR((F10+G10)*H10, 0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="2">
+      <c r="D10" s="29" t="s">
+        <v>98</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F10" s="29" t="s">
+        <v>99</v>
+      </c>
+      <c r="G10" s="29" t="s">
+        <v>105</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I10" s="35" t="s">
+        <v>104</v>
+      </c>
+      <c r="J10" s="29" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" s="7">
+        <v>1</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="D11" s="37">
+        <v>138.32</v>
+      </c>
+      <c r="E11" s="7">
+        <v>5</v>
+      </c>
+      <c r="F11" s="36">
+        <f>SUM(D11/E11)</f>
+        <v>27.663999999999998</v>
+      </c>
+      <c r="G11" s="36">
+        <v>60.17</v>
+      </c>
+      <c r="H11" s="7">
+        <v>1</v>
+      </c>
+      <c r="I11" s="14">
+        <v>340</v>
+      </c>
+      <c r="J11" s="14">
+        <f ca="1">(F11+G11/E11)*Заказы!$L$2+I11/E11</f>
+        <v>190.16265540000001</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" s="4">
+        <v>2</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="D12" s="37">
+        <v>274.17</v>
+      </c>
+      <c r="E12" s="7">
+        <v>50</v>
+      </c>
+      <c r="F12" s="36">
+        <f t="shared" ref="F12" si="2">SUM(D12/E12)</f>
+        <v>5.4834000000000005</v>
+      </c>
+      <c r="G12" s="36">
+        <v>43.72</v>
+      </c>
+      <c r="H12" s="7">
+        <v>1</v>
+      </c>
+      <c r="I12" s="14">
+        <v>407</v>
+      </c>
+      <c r="J12" s="14">
+        <f ca="1">(F12+G12/E12)*Заказы!$L$2+I12/E12</f>
+        <v>27.70485794</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13" s="4">
         <v>3</v>
       </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2">
-        <f>IFERROR(D11/E11, 0)</f>
-        <v>0</v>
-      </c>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2">
-        <f>IFERROR((F11+G11)*H11, 0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="2">
-        <v>4</v>
-      </c>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2">
-        <f>IFERROR(D12/E12, 0)</f>
-        <v>0</v>
-      </c>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2">
-        <f>IFERROR((F12+G12)*H12, 0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="22" t="s">
+      <c r="B13" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="D13" s="37">
+        <v>283.99</v>
+      </c>
+      <c r="E13" s="7">
+        <v>50</v>
+      </c>
+      <c r="F13" s="36">
+        <v>56.39</v>
+      </c>
+      <c r="G13" s="36">
+        <v>43.72</v>
+      </c>
+      <c r="H13" s="7">
+        <v>1</v>
+      </c>
+      <c r="I13" s="14">
+        <v>419</v>
+      </c>
+      <c r="J13" s="14">
+        <f ca="1">(F13+G13/E13)*Заказы!$L$2+I13/E13</f>
+        <v>184.59973812000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A14" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="23"/>
-      <c r="C13" s="23"/>
-      <c r="D13" s="23"/>
-      <c r="E13" s="23"/>
-      <c r="F13" s="23"/>
-      <c r="G13" s="23"/>
-      <c r="H13" s="23"/>
-      <c r="I13" s="4">
-        <f>SUM(I9:I12)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="28" t="s">
+      <c r="B14" s="32"/>
+      <c r="C14" s="32"/>
+      <c r="D14" s="32"/>
+      <c r="E14" s="32"/>
+      <c r="F14" s="32"/>
+      <c r="G14" s="32"/>
+      <c r="H14" s="32"/>
+      <c r="I14" s="33"/>
+      <c r="J14" s="39">
+        <f ca="1">SUM(J11:J13)</f>
+        <v>402.46725146000006</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15" s="43" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="23"/>
-      <c r="C14" s="23"/>
-      <c r="D14" s="23"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="23"/>
-      <c r="H14" s="23"/>
-      <c r="I14" s="5">
-        <f>I7+I13</f>
-        <v>0</v>
+      <c r="B15" s="44"/>
+      <c r="C15" s="44"/>
+      <c r="D15" s="44"/>
+      <c r="E15" s="44"/>
+      <c r="F15" s="44"/>
+      <c r="G15" s="44"/>
+      <c r="H15" s="44"/>
+      <c r="I15" s="45"/>
+      <c r="J15" s="46">
+        <f ca="1">J14+I8</f>
+        <v>485.18925146000004</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A8:I8"/>
-    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="A14:I14"/>
+    <mergeCell ref="A15:I15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80360DCB-FF63-4D27-BD94-E6F499FDE08A}">
+  <dimension ref="A1:J18"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="72.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="29" t="s">
+        <v>96</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="29" t="s">
+        <v>97</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="29" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="4">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4">
+        <v>2896270</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="D3" s="30">
+        <v>122.42</v>
+      </c>
+      <c r="E3" s="4">
+        <v>10</v>
+      </c>
+      <c r="F3" s="30">
+        <f>SUM(D3/E3)</f>
+        <v>12.242000000000001</v>
+      </c>
+      <c r="G3" s="4">
+        <v>0</v>
+      </c>
+      <c r="H3" s="4">
+        <v>1</v>
+      </c>
+      <c r="I3" s="30">
+        <f>SUM(F3*H3+G3)</f>
+        <v>12.242000000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="4">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4">
+        <v>2896089</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="D4" s="30">
+        <v>91.3</v>
+      </c>
+      <c r="E4" s="4">
+        <v>10</v>
+      </c>
+      <c r="F4" s="30">
+        <f t="shared" ref="F4:F8" si="0">SUM(D4/E4)</f>
+        <v>9.129999999999999</v>
+      </c>
+      <c r="G4" s="4">
+        <v>0</v>
+      </c>
+      <c r="H4" s="4">
+        <v>1</v>
+      </c>
+      <c r="I4" s="30">
+        <f t="shared" ref="I4:I8" si="1">SUM(F4*H4+G4)</f>
+        <v>9.129999999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="4">
+        <v>3</v>
+      </c>
+      <c r="B5" s="31">
+        <v>2896238</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="D5" s="30">
+        <v>430.56</v>
+      </c>
+      <c r="E5" s="4">
+        <v>50</v>
+      </c>
+      <c r="F5" s="30">
+        <f t="shared" si="0"/>
+        <v>8.6112000000000002</v>
+      </c>
+      <c r="G5" s="4">
+        <v>0</v>
+      </c>
+      <c r="H5" s="4">
+        <v>1</v>
+      </c>
+      <c r="I5" s="30">
+        <f t="shared" si="1"/>
+        <v>8.6112000000000002</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="4">
+        <v>4</v>
+      </c>
+      <c r="B6" s="4">
+        <v>2896131</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="D6" s="30">
+        <v>72.62</v>
+      </c>
+      <c r="E6" s="4">
+        <v>10</v>
+      </c>
+      <c r="F6" s="30">
+        <f t="shared" si="0"/>
+        <v>7.2620000000000005</v>
+      </c>
+      <c r="G6" s="4">
+        <v>0</v>
+      </c>
+      <c r="H6" s="4">
+        <v>1</v>
+      </c>
+      <c r="I6" s="30">
+        <f t="shared" si="1"/>
+        <v>7.2620000000000005</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" s="4">
+        <v>5</v>
+      </c>
+      <c r="B7" s="4">
+        <v>2896306</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="D7" s="30">
+        <v>540.88</v>
+      </c>
+      <c r="E7" s="4">
+        <v>10</v>
+      </c>
+      <c r="F7" s="30">
+        <f t="shared" si="0"/>
+        <v>54.088000000000001</v>
+      </c>
+      <c r="G7" s="4">
+        <v>0</v>
+      </c>
+      <c r="H7" s="4">
+        <v>1</v>
+      </c>
+      <c r="I7" s="30">
+        <f t="shared" si="1"/>
+        <v>54.088000000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" s="4">
+        <v>6</v>
+      </c>
+      <c r="B8" s="4">
+        <v>2896199</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D8" s="30">
+        <v>348.71</v>
+      </c>
+      <c r="E8" s="4">
+        <v>50</v>
+      </c>
+      <c r="F8" s="30">
+        <f t="shared" si="0"/>
+        <v>6.9741999999999997</v>
+      </c>
+      <c r="G8" s="4">
+        <v>0</v>
+      </c>
+      <c r="H8" s="4">
+        <v>2</v>
+      </c>
+      <c r="I8" s="30">
+        <f t="shared" si="1"/>
+        <v>13.948399999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" s="27"/>
+      <c r="B9" s="27"/>
+      <c r="C9" s="28"/>
+      <c r="D9" s="27"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
+      <c r="G9" s="27"/>
+      <c r="H9" s="27"/>
+      <c r="I9" s="7"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="23"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="39">
+        <f>SUM(I3:I9)</f>
+        <v>105.2816</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="34" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="34"/>
+      <c r="C11" s="34"/>
+      <c r="D11" s="34"/>
+      <c r="E11" s="34"/>
+      <c r="F11" s="34"/>
+      <c r="G11" s="34"/>
+      <c r="H11" s="34"/>
+      <c r="I11" s="34"/>
+      <c r="J11" s="34"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" s="29" t="s">
+        <v>98</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F12" s="29" t="s">
+        <v>99</v>
+      </c>
+      <c r="G12" s="29" t="s">
+        <v>105</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I12" s="35" t="s">
+        <v>104</v>
+      </c>
+      <c r="J12" s="29" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13" s="7">
+        <v>1</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="D13" s="37">
+        <v>297.18</v>
+      </c>
+      <c r="E13" s="7">
+        <v>5</v>
+      </c>
+      <c r="F13" s="36">
+        <f>SUM(D13/E13)</f>
+        <v>59.436</v>
+      </c>
+      <c r="G13" s="36">
+        <v>43.72</v>
+      </c>
+      <c r="H13" s="7">
+        <v>1</v>
+      </c>
+      <c r="I13" s="14">
+        <v>420</v>
+      </c>
+      <c r="J13" s="14">
+        <f ca="1">(F13+G13/E13)*Заказы!$L$2+I13/E13</f>
+        <v>293.81031400000006</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A14" s="4">
+        <v>2</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D14" s="37">
+        <v>117.31</v>
+      </c>
+      <c r="E14" s="7">
+        <v>50</v>
+      </c>
+      <c r="F14" s="36">
+        <f t="shared" ref="F14:F16" si="2">SUM(D14/E14)</f>
+        <v>2.3462000000000001</v>
+      </c>
+      <c r="G14" s="36">
+        <v>43.72</v>
+      </c>
+      <c r="H14" s="7">
+        <v>1</v>
+      </c>
+      <c r="I14" s="14">
+        <v>322</v>
+      </c>
+      <c r="J14" s="14">
+        <f ca="1">(F14+G14/E14)*Заказы!$L$2+I14/E14</f>
+        <v>16.350752380000003</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15" s="4">
+        <v>3</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="D15" s="37">
+        <v>274.17</v>
+      </c>
+      <c r="E15" s="7">
+        <v>50</v>
+      </c>
+      <c r="F15" s="36">
+        <f t="shared" si="2"/>
+        <v>5.4834000000000005</v>
+      </c>
+      <c r="G15" s="36">
+        <v>43.72</v>
+      </c>
+      <c r="H15" s="7">
+        <v>1</v>
+      </c>
+      <c r="I15" s="14">
+        <v>407</v>
+      </c>
+      <c r="J15" s="14">
+        <f ca="1">(F15+G15/E15)*Заказы!$L$2+I15/E15</f>
+        <v>27.70485794</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A16" s="4">
+        <v>4</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="D16" s="37">
+        <v>283.99</v>
+      </c>
+      <c r="E16" s="7">
+        <v>50</v>
+      </c>
+      <c r="F16" s="36">
+        <v>56.39</v>
+      </c>
+      <c r="G16" s="36">
+        <v>43.72</v>
+      </c>
+      <c r="H16" s="7">
+        <v>1</v>
+      </c>
+      <c r="I16" s="14">
+        <v>419</v>
+      </c>
+      <c r="J16" s="14">
+        <f ca="1">(F16+G16/E16)*Заказы!$L$2+I16/E16</f>
+        <v>184.59973812000001</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A17" s="32" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" s="32"/>
+      <c r="C17" s="32"/>
+      <c r="D17" s="32"/>
+      <c r="E17" s="32"/>
+      <c r="F17" s="32"/>
+      <c r="G17" s="32"/>
+      <c r="H17" s="32"/>
+      <c r="I17" s="33"/>
+      <c r="J17" s="39">
+        <f ca="1">SUM(J13:J16)</f>
+        <v>522.46566244000007</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A18" s="43" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18" s="44"/>
+      <c r="C18" s="44"/>
+      <c r="D18" s="44"/>
+      <c r="E18" s="44"/>
+      <c r="F18" s="44"/>
+      <c r="G18" s="44"/>
+      <c r="H18" s="44"/>
+      <c r="I18" s="45"/>
+      <c r="J18" s="40">
+        <f ca="1">J17+I10</f>
+        <v>627.7472624400001</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A11:J11"/>
+    <mergeCell ref="A18:I18"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C135D52-B6C5-4F8A-B597-7F31DFEF6A06}">
+  <dimension ref="A1:J11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="72.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="29" t="s">
+        <v>96</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="29" t="s">
+        <v>97</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="29" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="4">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4"/>
+      <c r="C3" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="D3" s="30">
+        <v>30</v>
+      </c>
+      <c r="E3" s="4">
+        <v>1</v>
+      </c>
+      <c r="F3" s="30">
+        <f>SUM(D3/E3)</f>
+        <v>30</v>
+      </c>
+      <c r="G3" s="4">
+        <v>0</v>
+      </c>
+      <c r="H3" s="4">
+        <v>1</v>
+      </c>
+      <c r="I3" s="30">
+        <f>SUM(F3*H3+G3)</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="4">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4"/>
+      <c r="C4" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="D4" s="30">
+        <v>30</v>
+      </c>
+      <c r="E4" s="4">
+        <v>1</v>
+      </c>
+      <c r="F4" s="30">
+        <f t="shared" ref="F4" si="0">SUM(D4/E4)</f>
+        <v>30</v>
+      </c>
+      <c r="G4" s="4">
+        <v>0</v>
+      </c>
+      <c r="H4" s="4">
+        <v>1</v>
+      </c>
+      <c r="I4" s="30">
+        <f t="shared" ref="I4" si="1">SUM(F4*H4+G4)</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="4">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4"/>
+      <c r="C5" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="D5" s="30">
+        <v>30</v>
+      </c>
+      <c r="E5" s="4">
+        <v>1</v>
+      </c>
+      <c r="F5" s="30">
+        <f t="shared" ref="F5" si="2">SUM(D5/E5)</f>
+        <v>30</v>
+      </c>
+      <c r="G5" s="4">
+        <v>0</v>
+      </c>
+      <c r="H5" s="4">
+        <v>1</v>
+      </c>
+      <c r="I5" s="30">
+        <f t="shared" ref="I5" si="3">SUM(F5*H5+G5)</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="23"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="23"/>
+      <c r="I6" s="39">
+        <f>SUM(I3:I4)</f>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="34" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="34"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="34"/>
+      <c r="E7" s="34"/>
+      <c r="F7" s="34"/>
+      <c r="G7" s="34"/>
+      <c r="H7" s="34"/>
+      <c r="I7" s="34"/>
+      <c r="J7" s="34"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D8" s="29" t="s">
+        <v>98</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F8" s="29" t="s">
+        <v>99</v>
+      </c>
+      <c r="G8" s="29" t="s">
+        <v>105</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I8" s="35" t="s">
+        <v>104</v>
+      </c>
+      <c r="J8" s="29" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" s="7">
+        <v>1</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="D9" s="37">
+        <v>210.42</v>
+      </c>
+      <c r="E9" s="7">
+        <v>5</v>
+      </c>
+      <c r="F9" s="36">
+        <f>SUM(D9/E9)</f>
+        <v>42.083999999999996</v>
+      </c>
+      <c r="G9" s="36">
+        <v>32.67</v>
+      </c>
+      <c r="H9" s="7">
+        <v>1</v>
+      </c>
+      <c r="I9" s="14">
+        <v>367</v>
+      </c>
+      <c r="J9" s="14">
+        <f ca="1">(F9+G9/E9)*Заказы!$L$2+I9/E9</f>
+        <v>223.0121714</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" s="32" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" s="32"/>
+      <c r="C10" s="32"/>
+      <c r="D10" s="32"/>
+      <c r="E10" s="32"/>
+      <c r="F10" s="32"/>
+      <c r="G10" s="32"/>
+      <c r="H10" s="32"/>
+      <c r="I10" s="33"/>
+      <c r="J10" s="39">
+        <f ca="1">SUM(J9:J9)</f>
+        <v>223.0121714</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" s="43" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="44"/>
+      <c r="C11" s="44"/>
+      <c r="D11" s="44"/>
+      <c r="E11" s="44"/>
+      <c r="F11" s="44"/>
+      <c r="G11" s="44"/>
+      <c r="H11" s="44"/>
+      <c r="I11" s="45"/>
+      <c r="J11" s="40">
+        <f ca="1">J10+I6</f>
+        <v>283.0121714</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A10:I10"/>
+    <mergeCell ref="A11:I11"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>